<commit_message>
fix(psi303): correct week 3 and 4 notes and teaching data
</commit_message>
<xml_diff>
--- a/data/psi303/PSI303-hafta3-uyku-kaygi.xlsx
+++ b/data/psi303/PSI303-hafta3-uyku-kaygi.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veri" sheetId="1" r:id="R2484c1d890a444a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yonerge" sheetId="2" r:id="R4644c79f0df74d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veri" sheetId="1" r:id="Rc7de1fbf8e0241e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yonerge" sheetId="2" r:id="Re6f6dc11d3da4c28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -303,7 +303,7 @@
   <x:sheetData>
     <x:row r="1" ht="27" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>katilimci_id</x:v>
+        <x:v>katilimci_kodu</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
         <x:v>uyku_saati</x:v>
@@ -323,7 +323,7 @@
         <x:v>K01</x:v>
       </x:c>
       <x:c r="B2" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C2" s="1" t="n">
         <x:v>4</x:v>
@@ -346,10 +346,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E3" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
@@ -357,7 +357,7 @@
         <x:v>K03</x:v>
       </x:c>
       <x:c r="B4" s="1" t="n">
-        <x:v>7.2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="1" t="n">
         <x:v>2</x:v>
@@ -366,7 +366,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E4" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
@@ -374,16 +374,16 @@
         <x:v>K04</x:v>
       </x:c>
       <x:c r="B5" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="1" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="n">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="E5" s="1" t="n">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
@@ -406,7 +406,7 @@
         <x:v>K06</x:v>
       </x:c>
       <x:c r="B7" s="1" t="n">
-        <x:v>25</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="1" t="n">
         <x:v>5</x:v>
@@ -423,7 +423,7 @@
         <x:v>K07</x:v>
       </x:c>
       <x:c r="B8" s="1" t="n">
-        <x:v>7</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C8" s="1" t="n">
         <x:v>3</x:v>
@@ -440,84 +440,16 @@
         <x:v>K08</x:v>
       </x:c>
       <x:c r="B9" s="1" t="n">
-        <x:v>5.9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C9" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E9" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="1" t="str">
-        <x:v>K09</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="n">
-        <x:v>8.6</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E10" s="1" t="n">
         <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="1" t="str">
-        <x:v>K10</x:v>
-      </x:c>
-      <x:c r="B11" s="1" t="n">
-        <x:v>6.8</x:v>
-      </x:c>
-      <x:c r="C11" s="1" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D11" s="1" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E11" s="1" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="1" t="str">
-        <x:v>K11</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="n">
-        <x:v>4.6</x:v>
-      </x:c>
-      <x:c r="C12" s="1" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="E12" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="1" t="str">
-        <x:v>K12</x:v>
-      </x:c>
-      <x:c r="B13" s="1" t="n">
-        <x:v>7.7</x:v>
-      </x:c>
-      <x:c r="C13" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D13" s="1" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E13" s="1" t="n">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -546,7 +478,7 @@
         <x:v>Kaynak</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>PSİ 303 ilk iki hafta öğretim paketindeki K01–K12 katılımcıları; Hafta 3 için uyku ve ders kaygısı sütunlarıyla genişletilmiş kurgusal tablo.</x:v>
+        <x:v>Ders notlarındaki K01–K08 sekiz kişilik kurgusal uyku/kaygı tablosu. Temizlik kopyasında K07 uyku_saati=25; K05 kaygi_m1 eksik.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -574,15 +506,15 @@
         <x:v>Görev 1</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>Ham veriyi koru. K06 uyku_saati=25 ile K05 kaygi_m1 boşluğunun farklı nedenlerini işlem günlüğüne yaz.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+        <x:v>Ham veriyi koru. K07 uyku_saati=25 ile K05 kaygi_m1 boşluğunun farklı nedenlerini işlem günlüğüne yaz.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>Görev 2</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>Kaynağı doğrulanamayan K06 uyku değerini analiz kopyasında eksik olarak işaretle; ham 25 değerini değiştirme.</x:v>
+        <x:v>Özgün kayıt erişilemez senaryosunda K07 uyku değerini yeni analiz sütununda eksik işaretle; ham 25 değerini koru. Doğrulanmış özgün kayıt varsa 6 saat ayrı gerekçeyle düzeltilebilir.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
@@ -593,12 +525,12 @@
         <x:v>kaygi_m3_ters = 6 - kaygi_m3 değişkenini oluştur. K01 ve K06 satırlarını elle kontrol et (m3 ters: 4 ve 5).</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9" ht="55" customHeight="1">
       <x:c r="A9" s="7" t="str">
         <x:v>Görev 4</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>Üç madde doluysa kaygi_toplam oluştur; eksik maddeli kaydı boş bırak. Tam puanlı katılımcıları filtrele.</x:v>
+        <x:v>Üç madde doluysa kaygi_toplam oluştur; K05 için eksik bırak. Tam kaygı puanlarını filtrele: n=8 → n=7. K07 kaygı analizinde kalır; uyku analizinde K07 eksiktir.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">

</xml_diff>